<commit_message>
Update meta-learning parameters and add new CSV files for SAVAGE loss function experiments
</commit_message>
<xml_diff>
--- a/table_meta_learning.xlsx
+++ b/table_meta_learning.xlsx
@@ -1,119 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erfanmirzaei/Projects/Generalization Bound/Gibbs-Generalization/data/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D45645C0-64B0-B840-8A29-50EB0FADD042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="5980" yWindow="2800" windowWidth="27240" windowHeight="16440" xr2:uid="{7D4AD33B-8E4B-E54B-9FA7-3099CBEA9477}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="5980" yWindow="2800" windowWidth="27240" windowHeight="16440" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
-  <si>
-    <t>CIFAR100 Classes</t>
-  </si>
-  <si>
-    <t>Mean SAVAGE training loss at beta = 128</t>
-  </si>
-  <si>
-    <t>Mean SAVAGE training loss at beta = 1000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mean SAVAGE training  loss at infinity </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mean SAVAGE test  loss at infinity </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mean 01 training  loss at infinity </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mean 01 test  loss at infinity </t>
-  </si>
-  <si>
-    <t>[0,1]</t>
-  </si>
-  <si>
-    <t>[2,50]</t>
-  </si>
-  <si>
-    <t>0.1350</t>
-  </si>
-  <si>
-    <t>0.0008</t>
-  </si>
-  <si>
-    <t>0.0906</t>
-  </si>
-  <si>
-    <t>0.0010</t>
-  </si>
-  <si>
-    <t>0.2542</t>
-  </si>
-  <si>
-    <t>0.2133</t>
-  </si>
-  <si>
-    <t>0.0012</t>
-  </si>
-  <si>
-    <t>0.4338</t>
-  </si>
-  <si>
-    <t>0.2232</t>
-  </si>
-  <si>
-    <t>0.2210</t>
-  </si>
-  <si>
-    <t>0.1324</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -132,21 +46,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -466,86 +439,169 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B42DA4F6-E0FF-B249-BB57-7EDF082BDCAE}">
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="28.33203125" customWidth="1"/>
-    <col min="6" max="6" width="32" customWidth="1"/>
-    <col min="7" max="7" width="34.83203125" customWidth="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="35.83203125" customWidth="1" min="3" max="3"/>
+    <col width="30.83203125" customWidth="1" min="4" max="4"/>
+    <col width="28.33203125" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="34.83203125" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>CIFAR100 Classes</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Mean SAVAGE training loss at beta = 128</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Mean SAVAGE training loss at beta = 1000</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mean SAVAGE training  loss at infinity </t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mean SAVAGE test  loss at infinity </t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mean 01 training  loss at infinity </t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mean 01 test  loss at infinity </t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" t="s">
-        <v>9</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>[0,1]</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0.2210</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0.1324</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0.0010</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0.0906</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.0008</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.1350</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" t="s">
-        <v>13</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>[2,50]</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0.4338</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0.2232</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0.0012</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.2133</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.0010</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.2542</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>[63,88]</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0.3817</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0.1943</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0.0002</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.2001</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0.2600</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add new CSV file for SAVAGE loss function test results with detailed parameters
</commit_message>
<xml_diff>
--- a/table_meta_learning.xlsx
+++ b/table_meta_learning.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -604,6 +604,43 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>[54,75]</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0.2144</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0.0740</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0.0544</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.0700</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add new CSV files for SAVAGE loss function test results and update meta-learning Excel file
</commit_message>
<xml_diff>
--- a/table_meta_learning.xlsx
+++ b/table_meta_learning.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -641,6 +641,80 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>[12,66]</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0.2170</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.1287</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.0011</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.1020</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.0010</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.1250</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>[40,72]</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0.3670</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0.1635</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>0.0002</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0.1798</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.2198</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update meta-learning parameters and add new CSV files for SAVAGE loss function test results
</commit_message>
<xml_diff>
--- a/table_meta_learning.xlsx
+++ b/table_meta_learning.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -715,6 +715,450 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>[60,97]</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0.1314</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0.0449</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0.0170</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.0250</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>[60,97]</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0.1314</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0.0449</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0.0170</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.0250</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>[48,67]</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0.2330</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>0.1241</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0.0021</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0.0795</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0.0020</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0.0959</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>[48,67]</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0.2330</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>0.1241</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0.0021</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0.0795</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0.0020</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0.0959</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>[23,81]</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0.2013</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>0.0871</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0.0794</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0.1050</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>[23,81]</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0.2013</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>0.0871</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>0.0794</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>0.1050</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>[14,52]</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0.1574</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>0.0487</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>0.0011</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>0.0374</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0.0010</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0.0550</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>[14,52]</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0.1574</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>0.0487</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>0.0011</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0.0374</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0.0010</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0.0550</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>[36,65]</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0.3387</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>0.1509</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0.0052</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0.1878</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.0050</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0.2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>[36,65]</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0.3387</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>0.1509</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>0.0052</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>0.1878</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0.0050</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0.2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>[26,57]</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0.3659</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>0.1669</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>0.0022</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0.1634</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0.0020</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>0.2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>[53,96]</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0.1355</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>0.0494</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>0.0021</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>0.0326</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>0.0020</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>0.0450</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add new test CSV files and update meta-learning parameters
- Created multiple new CSV files for test results with varying beta values and corresponding metrics.
- Updated the `meta_learning.py` script to increase the number of new pairs from 7 to 14 and changed the pair sampling seed from 82 to 92.
- Modified the `table_meta_learning.xlsx` file to reflect changes in the meta-learning setup.
</commit_message>
<xml_diff>
--- a/table_meta_learning.xlsx
+++ b/table_meta_learning.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1455,6 +1455,672 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>[8,29]</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0.3693</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>0.1653</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>0.0002</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>0.1805</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>0.2056</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>[82,89]</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0.2489</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>0.1152</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>0.0458</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>0.0550</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>[4,28]</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>0.2690</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>0.1259</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>0.1133</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>0.1350</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>[16,27]</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>0.3285</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>0.1696</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>0.1067</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>0.1252</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>[46,89]</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>0.3098</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>0.1398</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>0.0789</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0.0871</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>[20,25]</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>0.2381</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>0.1360</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>0.0027</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>0.1463</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>0.0025</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>0.1794</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>[33,38]</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>0.2552</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>0.1526</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>0.0011</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>0.1118</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>0.0010</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>0.1371</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>[17,39]</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>0.1736</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>0.0758</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>0.0587</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>0.0800</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>[31,69]</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0.1663</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>0.0740</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>0.0050</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>0.0584</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>0.0050</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>0.0745</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>[3,62]</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>0.2129</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>0.0874</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>0.0665</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>0.0850</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>[59,86]</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>0.2341</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>0.1062</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>0.0011</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>0.0871</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>0.0010</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>0.0950</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>[29,68]</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>0.1827</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>0.0718</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>0.0011</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>0.0567</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>0.0010</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>0.0700</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>[80,92]</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>0.2798</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>0.1458</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>0.0021</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>0.1050</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>0.0020</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>0.1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>[30,73]</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>0.3946</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>0.2154</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>0.0033</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>0.2442</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>0.0030</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>0.2800</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>[28,49]</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>0.1442</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>0.0555</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>0.0354</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>0.0364</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>[35,46]</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>0.4080</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>0.2684</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>0.0003</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>0.2589</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>0.3402</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>[34,99]</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>0.3442</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>0.1562</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>0.0012</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>0.0966</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>0.0010</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>0.1201</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>[13,51]</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>0.2739</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>0.1349</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>0.0011</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>0.0926</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>0.0010</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>0.1150</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add new CSV files for SAVAGE loss function experiments with varying beta values
- Created multiple CSV files containing results from experiments using the SAVAGE loss function on the CIFAR-100 dataset.
- Each file includes metrics such as BCE Train/Test, EMA losses, and gradient norms for different beta values.
- Summary sections detail the parameters used in each experiment, including device, network architecture, dataset specifics, and training configurations.
</commit_message>
<xml_diff>
--- a/table_meta_learning.xlsx
+++ b/table_meta_learning.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2121,6 +2121,154 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>[9,91]</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>0.2946</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>0.1266</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>0.0011</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>0.0987</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>0.0010</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>0.1250</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>[24,61]</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>0.1694</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>0.0849</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>0.0022</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>0.0592</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>0.0020</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>0.0718</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>[15,58]</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>0.3584</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>0.1578</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>0.0011</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>0.1183</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>0.0010</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>0.1400</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>[5,64]</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>0.2742</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>0.1559</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>0.1471</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>0.1850</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add new test CSV files for SAVAGE loss function with updated parameters
</commit_message>
<xml_diff>
--- a/table_meta_learning.xlsx
+++ b/table_meta_learning.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2269,6 +2269,80 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>[5,77]</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>0.3389</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>0.1482</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>0.1286</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>0.1693</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>[24,95]</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>0.1554</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>0.0726</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>0.0646</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>0.0700</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>